<commit_message>
docs: record Day 2 Docker baseline and learning outcomes
</commit_message>
<xml_diff>
--- a/FabFlow_K8s_30天進度表.xlsx
+++ b/FabFlow_K8s_30天進度表.xlsx
@@ -153,7 +153,7 @@
       </c>
       <c r="B6" s="2">
         <f>COUNTIF('每日進度'!I2:I31,"已完成")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
@@ -164,7 +164,7 @@
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('每日進度'!I2:I31,"已完成")/30</f>
-        <v>0</v>
+        <v>0.06666666666666667</v>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
@@ -429,7 +429,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -439,7 +439,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/k8s/day01-architecture.md；依使用者確認已完成</t>
         </is>
       </c>
     </row>
@@ -482,7 +482,7 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
@@ -492,7 +492,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/k8s/day02-docker-baseline.md；Compose healthy、HTTP smoke 全部 PASS；使用者確認兩種情境 KPI 與 refresh 成功</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: deploy API to kind and record Day 3–4 learning notes
</commit_message>
<xml_diff>
--- a/FabFlow_K8s_30天進度表.xlsx
+++ b/FabFlow_K8s_30天進度表.xlsx
@@ -153,7 +153,7 @@
       </c>
       <c r="B6" s="2">
         <f>COUNTIF('每日進度'!I2:I31,"已完成")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
@@ -164,7 +164,7 @@
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('每日進度'!I2:I31,"已完成")/30</f>
-        <v>0.06666666666666667</v>
+        <v>0.1333333333333333</v>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
@@ -535,7 +535,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -545,7 +545,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/k8s/day03-local-cluster.md；kind-fabflow 節點 Ready；測試 Pod exec 與刪除驗收通過；重建指令已記錄，未實測重建</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
@@ -598,7 +598,7 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/k8s/day04-api.md；Deployment 1/1、Pod Running；port-forward readiness 與 Swagger 驗收通過</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: deploy dashboard and record Day 5 learning notes
</commit_message>
<xml_diff>
--- a/FabFlow_K8s_30天進度表.xlsx
+++ b/FabFlow_K8s_30天進度表.xlsx
@@ -153,7 +153,7 @@
       </c>
       <c r="B6" s="2">
         <f>COUNTIF('每日進度'!I2:I31,"已完成")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
@@ -164,7 +164,7 @@
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('每日進度'!I2:I31,"已完成")/30</f>
-        <v>0.1333333333333333</v>
+        <v>0.1666666666666667</v>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
@@ -641,7 +641,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -651,7 +651,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/k8s/day05-dashboard.md；Dashboard 部署、ConfigMap、Service DNS、兩情境 KPI load/refresh 與觀念問答通過</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add health probes and resource settings with Day 6 notes
</commit_message>
<xml_diff>
--- a/FabFlow_K8s_30天進度表.xlsx
+++ b/FabFlow_K8s_30天進度表.xlsx
@@ -153,7 +153,7 @@
       </c>
       <c r="B6" s="2">
         <f>COUNTIF('每日進度'!I2:I31,"已完成")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
@@ -164,7 +164,7 @@
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('每日進度'!I2:I31,"已完成")/30</f>
-        <v>0.1666666666666667</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
@@ -694,7 +694,7 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
@@ -704,7 +704,7 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/k8s/day06-health-resources.md；probes、requests、limits 生效；兩服務 Ready、UI 驗收與問答通過，重啟 0 次；EndpointSlice 未另提供輸出</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: record Day 7 troubleshooting and recovery outcomes
</commit_message>
<xml_diff>
--- a/FabFlow_K8s_30天進度表.xlsx
+++ b/FabFlow_K8s_30天進度表.xlsx
@@ -153,7 +153,7 @@
       </c>
       <c r="B6" s="2">
         <f>COUNTIF('每日進度'!I2:I31,"已完成")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
@@ -164,7 +164,7 @@
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('每日進度'!I2:I31,"已完成")/30</f>
-        <v>0.2</v>
+        <v>0.2333333333333333</v>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
@@ -747,7 +747,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -757,7 +757,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/k8s/day07-debugging.md；Service targetPort、API URL 故障定位與修復通過；補記 value/valueFrom 衝突；UI 恢復與問答通過</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add Day 11 PostgreSQL result writes and verification records
</commit_message>
<xml_diff>
--- a/FabFlow_K8s_30天進度表.xlsx
+++ b/FabFlow_K8s_30天進度表.xlsx
@@ -153,7 +153,7 @@
       </c>
       <c r="B6" s="2">
         <f>COUNTIF('每日進度'!I2:I31,"已完成")</f>
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
@@ -164,7 +164,7 @@
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('每日進度'!I2:I31,"已完成")/30</f>
-        <v>0.2333333333333333</v>
+        <v>0.36666666666666664</v>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
@@ -800,7 +800,7 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
@@ -810,7 +810,7 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/k8s/day08-rebuild.md；核心操作驗收完成：namespace 重建、舊 run 回 404、新 baseline 與 UI KPI 通過；Service DNS／selector 觀念已補充。保留既有 cluster 與映像，非空白節點重建；實際時數待填。</t>
         </is>
       </c>
     </row>
@@ -853,7 +853,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/k8s/day09-storage-design.md；儲存介面、PostgreSQL schema 與逐步觀念練習完成；定義完整結果提交後才回 201、查無與故障區分及 API 契約；本課為設計，尚未實作儲存介面；實際時數待填。</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/k8s/day10-postgres-dev.md；Compose PostgreSQL 17、具名 volume、schema 初始化與敏感設定完成；使用者輸出確認 API 容器可連 DB 並查到 completed_runs；結果仍存記憶體，尚未實作 DB 寫入／查詢及結果持久化驗收；實際時數待填。</t>
         </is>
       </c>
     </row>
@@ -959,7 +959,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/k8s/day11-postgres-write.md；儲存介面與 PostgreSQL save 完成；真實 DB 完整 JSON 比對、注入測試 API 的 HTTP 201／故障 503 通過；181 tests passed。正式 API 仍使用記憶體，adapter 缺 get，查詢與正式切換留 Day 12；實際時數待填。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add Day 12 PostgreSQL queries and persistence acceptance
</commit_message>
<xml_diff>
--- a/FabFlow_K8s_30天進度表.xlsx
+++ b/FabFlow_K8s_30天進度表.xlsx
@@ -153,7 +153,7 @@
       </c>
       <c r="B6" s="2">
         <f>COUNTIF('每日進度'!I2:I31,"已完成")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
@@ -164,7 +164,7 @@
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('每日進度'!I2:I31,"已完成")/30</f>
-        <v>0.36666666666666664</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
@@ -1022,7 +1022,7 @@
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/k8s/day12-postgres-read.md；PostgreSQL get、Compose 後端切換完成；API 重啟完整結果一致、未知 ID 三端點 404、真實 DB 停止三端點 503、DB 重建沿用 volume 後資料一致；外接 SSD 掛載錯誤於 Docker Desktop 重啟後排除，根因未確認。腳本 prepare/verify 實測通過，unavailable 未執行；184 tests passed；實際時數待填。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: deploy PostgreSQL on Kubernetes and verify API pod persistence
</commit_message>
<xml_diff>
--- a/FabFlow_K8s_30天進度表.xlsx
+++ b/FabFlow_K8s_30天進度表.xlsx
@@ -153,7 +153,7 @@
       </c>
       <c r="B6" s="2">
         <f>COUNTIF('每日進度'!I2:I31,"已完成")</f>
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
@@ -164,7 +164,7 @@
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('每日進度'!I2:I31,"已完成")/30</f>
-        <v>0.4</v>
+        <v>0.43333333333333335</v>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1075,7 +1075,7 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/k8s/day13-postgres-pvc.md；K8s PostgreSQL 17 單副本、1Gi PVC Bound、Secret、SQL ConfigMap、Service 與 API day13 映像部署完成；API Pod 重建後三份結果與外部快照一致，未知 ID 三端點 404；184 tests passed，server dry run 通過。DB 非 HA；DB Pod 重建未實測，本機 PVC 不保護整個 cluster 刪除；實際時數待填。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: verify dual API replicas and database outage recovery
</commit_message>
<xml_diff>
--- a/FabFlow_K8s_30天進度表.xlsx
+++ b/FabFlow_K8s_30天進度表.xlsx
@@ -153,7 +153,7 @@
       </c>
       <c r="B6" s="2">
         <f>COUNTIF('每日進度'!I2:I31,"已完成")</f>
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
@@ -164,7 +164,7 @@
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('每日進度'!I2:I31,"已完成")/30</f>
-        <v>0.43333333333333335</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/k8s/day14-api-replicas.md；API replicas=2；Pod A 建立 run，兩個具名 Pod 各自 HTTP 查詢 summary、metrics、events 與同一快照一致，未知 ID 三端點皆 404；兩個 psycopg 連線確認同一 PostgreSQL server 與資料列。184 tests passed、API server dry run 通過。兩 API 同節點、DB 單副本，非 HA／效能驗證；實際時數待填。</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -1181,7 +1181,7 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/k8s/day15-persistence-acceptance.md；兩 API 基線通過，K8s DB 縮為 0 後已知／未知 GET 均 503，兩 POST 均 503 且無 Location；DB 新 Pod 沿用原 PVC 恢復後舊結果一致、失敗 scenario 各 0 列、新 POST 201。184 tests passed、全目錄 server dry run 通過。中途終止 API 僅觀念確認，未實測；無自動續跑／重試；實際時數待填。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add Helm chart and verify installation and upgrades
</commit_message>
<xml_diff>
--- a/FabFlow_K8s_30天進度表.xlsx
+++ b/FabFlow_K8s_30天進度表.xlsx
@@ -153,7 +153,7 @@
       </c>
       <c r="B6" s="2">
         <f>COUNTIF('每日進度'!I2:I31,"已完成")</f>
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
@@ -164,7 +164,7 @@
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('每日進度'!I2:I31,"已完成")/30</f>
-        <v>0.5</v>
+        <v>0.5666666666666667</v>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
@@ -1234,7 +1234,7 @@
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/k8s/day16-helm-skeleton.md；Helm v4.3.1、Chart.yaml/values/templates 骨架完成；lint 通過（icon INFO），完整渲染 3 Deployments＋3 Services，API 副本與 image tag 覆寫通過。184 tests passed，品質檢查通過。尚未安裝 chart；連線、Secret/PVC、初始化、probes/resources 留 Day 17；實際時數待填。</t>
         </is>
       </c>
     </row>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/k8s/day17-helm-install-upgrade.md；chart 補連線、ConfigMap、外部 Secret 引用、初始化/PVC、probes/resources；乾淨 fabflow-helm namespace 安裝 revision1，兩情境 HTTP 驗收通過；API 2→1 revision2、reset恢復2 revision3，完整結果一致，新 Pod 查詢通過。184 tests passed、SQL cmp/lint/server dry run 通過。chart0.1.0、單DB，本課未測image更新或零停機；實際時數待填。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: record Day 18 image CI acceptance
</commit_message>
<xml_diff>
--- a/FabFlow_K8s_30天進度表.xlsx
+++ b/FabFlow_K8s_30天進度表.xlsx
@@ -153,7 +153,7 @@
       </c>
       <c r="B6" s="2">
         <f>COUNTIF('每日進度'!I2:I31,"已完成")</f>
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
@@ -164,7 +164,7 @@
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('每日進度'!I2:I31,"已完成")/30</f>
-        <v>0.5666666666666667</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
@@ -1330,7 +1330,7 @@
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/k8s/day18-image-ci.md；PR #1 使用者確認四個 CI jobs 成功；API/Dashboard 建置日誌確認同 SHA 45160aa86a58c4bdb4592d08addc655dc664e454。images needs quality/containers，matrix targets 與 SHA tags 完成。映像僅在 runner，未發布 registry／部署／確認合併；實際時數待填。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: finalize Day 18 CI and merge records
</commit_message>
<xml_diff>
--- a/FabFlow_K8s_30天進度表.xlsx
+++ b/FabFlow_K8s_30天進度表.xlsx
@@ -1340,7 +1340,7 @@
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>docs/k8s/day18-image-ci.md；PR #1 使用者確認四個 CI jobs 成功；API/Dashboard 建置日誌確認同 SHA 45160aa86a58c4bdb4592d08addc655dc664e454。images needs quality/containers，matrix targets 與 SHA tags 完成。映像僅在 runner，未發布 registry／部署／確認合併；實際時數待填。</t>
+          <t>docs/k8s/day18-image-ci.md；Day 18 完成。PR #1 四項 CI 與紀錄提交 8421b3d 更新均依使用者確認成功；雙映像 PR SHA 45160aa86a58c4bdb4592d08addc655dc664e454。PR 已合併，main/origin/main 0e16ef4，main push 四項 CI 亦依使用者確認成功。映像僅在 runner，未發布／部署；手動觸發未驗證；實際時數待填。</t>
         </is>
       </c>
     </row>
@@ -1393,7 +1393,7 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>尚未開始操作。下一步先核對主機／kind 節點架構、工作目錄與 live cluster，再選擇映像保存／取得方式，讓 Helm 使用指定 commit 版本；已提出架構查詢指令，尚無使用者輸出。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: pin kind deployment images and record Day 19 acceptance
</commit_message>
<xml_diff>
--- a/FabFlow_K8s_30天進度表.xlsx
+++ b/FabFlow_K8s_30天進度表.xlsx
@@ -153,7 +153,7 @@
       </c>
       <c r="B6" s="2">
         <f>COUNTIF('每日進度'!I2:I31,"已完成")</f>
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
@@ -164,7 +164,7 @@
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('每日進度'!I2:I31,"已完成")/30</f>
-        <v>0.6</v>
+        <v>0.6333333333333333</v>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>尚未開始操作。下一步先核對主機／kind 節點架構、工作目錄與 live cluster，再選擇映像保存／取得方式，讓 Helm 使用指定 commit 版本；已提出架構查詢指令，尚無使用者輸出。</t>
+          <t>docs/k8s/day19-versioned-deployment.md；本機 ARM64 從乾淨 commit 395df1ec02a010163ea46e68374feb607c0c39bd 建置雙映像並載入 kind；values-kind.yaml 固定 SHA，lint/template 通過。Helm revision4 deployed、雙API/Dashboard新Pod版本正確，DB/PVC不變；舊結果快照三份一致、未知ID404，兩情境HTTP smoke全PASS。未發布registry／量測更新失敗率／rollback；待提交與PR CI，實際時數待填。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: record Day 20 rolling update measurements
</commit_message>
<xml_diff>
--- a/FabFlow_K8s_30天進度表.xlsx
+++ b/FabFlow_K8s_30天進度表.xlsx
@@ -153,7 +153,7 @@
       </c>
       <c r="B6" s="2">
         <f>COUNTIF('每日進度'!I2:I31,"已完成")</f>
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
@@ -164,7 +164,7 @@
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('每日進度'!I2:I31,"已完成")/30</f>
-        <v>0.6333333333333333</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
@@ -1436,7 +1436,7 @@
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t/>
+          <t>docs/k8s/day20-rolling-update.md；API SHA 794dbaafc1697a8812358b30b0808c6100242ebe、明確RollingUpdate 1/0；Helm revision5成功6.818秒。固定Dashboard經Service探測300秒、2376請求5失敗（3拒絕連線2逾時），非零停機，根因未確認；舊三份結果一致、未知ID404，新API 2/2 Ready，Dashboard/DB不變。原始紀錄artifacts/day20；待提交/PR CI，實際時數待填。</t>
         </is>
       </c>
     </row>

</xml_diff>